<commit_message>
Show example transactions as debit and credit journal entries
</commit_message>
<xml_diff>
--- a/samples/새회사변환예제/02_노바부품_시산표_통제자료.xlsx
+++ b/samples/새회사변환예제/02_노바부품_시산표_통제자료.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="R98482cef3e1540d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시산표" sheetId="2" r:id="R104638c55e154e4b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="독립통제" sheetId="3" r:id="R7df7ae0821d6405c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="감사조정" sheetId="4" r:id="Rcb6f91ba5e7c4861"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모듈연결" sheetId="5" r:id="R534ccac1b3f144c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="설정" sheetId="1" r:id="R9c6cb1a59a5b4066"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="시산표" sheetId="2" r:id="R4c72303c301c40ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="독립통제" sheetId="3" r:id="R4b8e32ea0a1844a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="감사조정" sheetId="4" r:id="Rff054883ad0b4519"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="모듈연결" sheetId="5" r:id="R15a96cc8d5b94436"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -389,7 +389,7 @@
         <x:v>001101</x:v>
       </x:c>
       <x:c r="C2" s="2" t="str">
-        <x:v>국민보통예금</x:v>
+        <x:v>국민은행</x:v>
       </x:c>
       <x:c r="D2" s="7" t="n">
         <x:v>0</x:v>
@@ -412,7 +412,7 @@
         <x:v>001102</x:v>
       </x:c>
       <x:c r="C3" s="2" t="str">
-        <x:v>신한당좌예금</x:v>
+        <x:v>신한은행</x:v>
       </x:c>
       <x:c r="D3" s="7" t="n">
         <x:v>0</x:v>
@@ -458,7 +458,7 @@
         <x:v>001301</x:v>
       </x:c>
       <x:c r="C5" s="2" t="str">
-        <x:v>상품재고</x:v>
+        <x:v>재고자산</x:v>
       </x:c>
       <x:c r="D5" s="7" t="n">
         <x:v>0</x:v>
@@ -527,7 +527,7 @@
         <x:v>005101</x:v>
       </x:c>
       <x:c r="C8" s="2" t="str">
-        <x:v>상품매출원가</x:v>
+        <x:v>매출원가</x:v>
       </x:c>
       <x:c r="D8" s="7" t="n">
         <x:v>0</x:v>

</xml_diff>